<commit_message>
fix: restore Verified_Partners data wiped by the cron bug
The 4x cron ran generate_partner_sourcing.py before the previous
commit's fix landed, and its Verified_Partners-destroying ExcelWriter
call wiped the 3 real Japan leads (Tsukuino, Pesca K&M, True World
Japan) from the live abalone_buyers_leads.xlsx and the corresponding
section of Abalone_Buyers_Lead_List.md. Restored both from the
last-known-good version (078ea5a) and regenerated the report with the
now-fixed script to confirm the section renders correctly and survives
another run.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BIZ-Jeonbok/data/abalone_buyers_leads.xlsx
+++ b/BIZ-Jeonbok/data/abalone_buyers_leads.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sourcing_Candidates" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sourcing_History" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sourcing_Candidates" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified_Partners" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sourcing_History" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +36,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +44,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,67 +419,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>국가 (Country)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>데이터 수집일</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>EDA 데이터 근거 (HS Code별 순위/수입액/물량)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>후보 HS Code 수</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>최고 순위</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>우선순위 점수</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>조사 상태</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>후보 파트너/에이전트명</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>회사 이메일</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>웹사이트 / LinkedIn</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Messenger</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>본사 위치</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>비고/메모</t>
         </is>
@@ -504,7 +493,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -541,7 +530,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -578,7 +567,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -615,7 +604,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -660,7 +649,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -697,7 +686,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -734,7 +723,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -771,7 +760,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -808,7 +797,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -845,7 +834,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -882,7 +871,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -919,7 +908,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -956,7 +945,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -993,7 +982,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1030,7 +1019,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1067,7 +1056,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1104,7 +1093,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1141,7 +1130,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1178,7 +1167,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1215,7 +1204,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1252,7 +1241,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1289,7 +1278,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-31 11:28:57</t>
+          <t>2026-07-31 21:06:19</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1329,44 +1318,356 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>수집 구동 시기 (Execution Timestamp)</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>참조 HS Code 표 수</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>이번 실행 발견 국가 수</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>신규 후보국 수 (New)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>누적 총 후보국 수 (Total Accumulated)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>상태 (Status)</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>조사일 (Research Date)</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>국가 (Country)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>회사명/에이전트명</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>구분 (법인/개인 에이전트)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>이메일</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>웹사이트 / LinkedIn URL</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Messenger/연락처</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>조사 범위 (HS Code 표)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>본사 위치 (상세)</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>주요 취급 품목 및 특징</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>잠재적 협력 포인트</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>출처 URL (검증 근거)</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>비고</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>2026-07-31 14:58:21</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Pesca K &amp; M Co., Ltd.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>법인</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>pescauno@nifty.com</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://www.trade-seafood.com/directory/seafood/exporters/pesca-k-m-co-japan.htm</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Tel: +81 3 5633 8765 / Fax: +81 3 5633 8766 (담당자: Hiro Kikuchi, Manager)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>표2 (HS 160557)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Tokyo</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Sun East Bldg. 3F, 3-14-17 Toyo, Koto-Ku, 135-0016 (칠레/페루 지사보유)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>칠레/페루산 수산물 수입업체. 칠레산 냉동 대하(각질포함), 통조림 대하(4-10조각/tin 213g), 건조 대하를 다룴. 브랜드: Pesca Uno, Don Jorge, Compomar.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>통조림/건조 전복 가공품 유통 실적이 있는 수입상 — 한국산 가공품(HS160557) 종류 확장 제안 가능성.</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>https://www.trade-seafood.com/directory/seafood/exporters/pesca-k-m-co-japan.htm</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>페이지에 표시된 이메일은 JS 난독화(자동 추출 불가) 처리되어 있어 실제 주소로 기록하지 않음. 전화/팩스로 연락 권장.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-31 14:58:21</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>True World Japan Inc.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>법인</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://www.trueworld-jp.com/en/product/awabi/index.html</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Tel: 03-6859-0881 (본사) / 03-6204-9532 (도쿄 지사)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>표1 (HS 030781)</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Tokyo</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Shinmei Bldg. 3F, 3-3 Akashi-cho, Chuo-ku 104-0044 (본사); 후쿠오카 지사도 보유</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>한국 완도산 전복(Wando abalone)을 명시적으로 취급 중 — Live/Boiled/Frozen 규격별(50g~110g) 판매.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>이미 한국산(완도) 전복을 수입·판매 중인 실적이 있는 트레이딩 회사 — 신규 한국 공급처로서 가장 직접적인 협력 가능성.</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>https://www.trueworld-jp.com/en/product/awabi/index.html</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>공개 이메일 없음, 웹사이트 문의폼/대표번호를 통한 컸택 권장.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-31 14:58:21</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Tsukuino Co. Ltd.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>법인</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>tukuino@heart.ocn.ne.jp</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://www.tsukuino.com/english.html</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>표1 (HS 030781)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Tokyo</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Toyosu Market, store 1065-1068, Koto-ku</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>1965년 설립. Toyosu Market 소재 수산물 도매상. 활어, 전복(abalone), 신선어, 냉동품, 가공품, 건어물 등 취급.</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>전복을 포함한 다양한 수산물을 이미 취급 중인 도매상 — 국가/희망 어종/예상 물량을 포함해 연락 요망.</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>https://www.tsukuino.com/english.html</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>이메일만 공개, 전화번호/문의폼 없음.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>수집 구동 시기 (Execution Timestamp)</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>참조 HS Code 표 수</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>이번 실행 발견 국가 수</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>신규 후보국 수 (New)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>누적 총 후보국 수 (Total Accumulated)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>상태 (Status)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>2026-07-31 13:55:51</t>
         </is>
       </c>
@@ -1407,6 +1708,30 @@
         <v>22</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>정상 완료 (Success)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-31 21:06:19</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>22</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>22</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>정상 완료 (Success)</t>
         </is>

</xml_diff>